<commit_message>
docs: completa i dati del gruppo nel pacchetto
</commit_message>
<xml_diff>
--- a/deliverables/BiblioFlow-CR-BF-01-consegna-2026-10-13/02.Informazioni progetto ISTA - BiblioFlow.xlsx
+++ b/deliverables/BiblioFlow-CR-BF-01-consegna-2026-10-13/02.Informazioni progetto ISTA - BiblioFlow.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="progetto" sheetId="1" r:id="R71cd4a39235342a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partecipanti" sheetId="2" r:id="R12a724d99e3941b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="progetto" sheetId="1" r:id="R81b731a548f54cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="partecipanti" sheetId="2" r:id="R037919bbc95648c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30,9 +30,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Email unisa</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Noma Progetto</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -621,22 +618,22 @@
       <x:c r="D1" s="5" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="s">
-        <x:v>7</x:v>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Nome Progetto</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="11" t="str">
-        <x:v>0512117090</x:v>
+        <x:v>NF22500193</x:v>
       </x:c>
       <x:c r="B2" s="12" t="str">
-        <x:v>Mancino</x:v>
+        <x:v>Celzo</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>Renato</x:v>
+        <x:v>Mario</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
-        <x:v>r.mancino10@studenti.unisa.it</x:v>
+        <x:v>m.celzo@studenti.unisa.it</x:v>
       </x:c>
       <x:c r="E2" s="12" t="str">
         <x:v>BiblioFlow</x:v>
@@ -644,24 +641,24 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
-        <x:v>0512118665</x:v>
+        <x:v>NF22500242</x:v>
       </x:c>
       <x:c r="B3" s="12" t="str">
-        <x:v>Celzo</x:v>
+        <x:v>Mancino</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>Mario</x:v>
+        <x:v>Renato</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
-        <x:v>m.celzo@studenti.unisa.it</x:v>
+        <x:v>r.mancino10@studenti.unisa.it</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
         <x:v>BiblioFlow</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="14" t="str">
-        <x:v>DA CONFERMARE</x:v>
+      <x:c r="A4" s="11" t="str">
+        <x:v>NF22500210</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
         <x:v>Ferrara</x:v>
@@ -669,8 +666,8 @@
       <x:c r="C4" s="12" t="str">
         <x:v>Alfonso Maria</x:v>
       </x:c>
-      <x:c r="D4" s="16" t="str">
-        <x:v>DA CONFERMARE</x:v>
+      <x:c r="D4" s="12" t="str">
+        <x:v>a.ferrara198@studenti.unisa.it</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
         <x:v>BiblioFlow</x:v>

</xml_diff>